<commit_message>
feat/new corrections and final document
</commit_message>
<xml_diff>
--- a/Plantillas/PlantillaDocumentaciónDiagramaComponentes.xlsx
+++ b/Plantillas/PlantillaDocumentaciónDiagramaComponentes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28908"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29910"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Luciana\Documents\Estructura\1. Artefactos proyecto\1.2. Artefactos técnicos\1.2.2. Diseño detallado\1.2.2.2. Diagrama de componentes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="77" documentId="13_ncr:101_{4574D783-3C4B-4454-AA23-2FEE293D4EC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E9BD7DE-EA86-44C2-A32B-CD47BC847BDD}"/>
+  <xr:revisionPtr revIDLastSave="141" documentId="13_ncr:101_{4574D783-3C4B-4454-AA23-2FEE293D4EC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7F7B760-4F82-4815-8FCC-A0B7A4081C2B}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" firstSheet="1" xr2:uid="{89DBD8A5-DC87-4190-9617-E764C549D606}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" xr2:uid="{89DBD8A5-DC87-4190-9617-E764C549D606}"/>
   </bookViews>
   <sheets>
     <sheet name="Diagrama Componentes" sheetId="7" r:id="rId1"/>
@@ -126,13 +126,13 @@
     <t>Permite gestionar de forma organizada las solicitudes de cotizacion generadas por los clientes.</t>
   </si>
   <si>
-    <t>Aplicación Móvil</t>
+    <t>Aplicación Web</t>
   </si>
   <si>
     <t>Interfaz gráfica que permite a los usuarios interactuar con las funcionalidades del sistema a través de servicios REST API.</t>
   </si>
   <si>
-    <t>Ofrece una experiencia intuitiva para que el usuario pueda realizar gestiones fácilmente desde su dispositivo móvil.</t>
+    <t>Ofrece una experiencia intuitiva para que el usuario pueda realizar gestiones fácilmente desde un navegador web.</t>
   </si>
   <si>
     <t>Servicios REST API de cada módulo</t>
@@ -280,8 +280,6 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -291,6 +289,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -322,25 +322,23 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>457200</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>695325</xdr:colOff>
-      <xdr:row>74</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="0" cy="0"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2">
+        <xdr:cNvPr id="51" name="Imagen 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9A4B61D5-D313-BBE0-14A8-7E5377CE4971}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F4774D0D-E5B6-2C7B-60FB-9F665DC5B01C}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{965E4120-1660-6D7D-A918-A2E229481652}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -356,8 +354,55 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="457200" y="438150"/>
-          <a:ext cx="22431375" cy="13735050"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>923925</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D583469-087C-D7C5-1FDC-BC24843BA15C}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{F4774D0D-E5B6-2C7B-60FB-9F665DC5B01C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="923925" y="914400"/>
+          <a:ext cx="5495925" cy="3381375"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -669,17 +714,17 @@
   <dimension ref="A2:O9"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="11.42578125" style="5"/>
+    <col min="1" max="1" width="24.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="11.42578125" style="8"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:15">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:15">
-      <c r="O9" s="6"/>
+      <c r="O9" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -733,7 +778,7 @@
       <c r="E3" s="11"/>
     </row>
     <row r="4" spans="1:8" s="2" customFormat="1">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="5" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="3" t="s">
@@ -750,122 +795,122 @@
       </c>
     </row>
     <row r="5" spans="1:8" ht="45.75">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="6" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="45.75">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="6" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="30.75">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="6" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="30.75">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="6" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="45.75">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="6" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="45.75">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H10" s="9"/>
+      <c r="H10" s="7"/>
     </row>
     <row r="11" spans="1:8" ht="76.5">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="6" t="s">
         <v>36</v>
       </c>
     </row>
@@ -881,19 +926,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="36cf0646-7300-4608-bcc3-e29ed014863a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="734bc881-a844-4d86-9741-49f87248cc41" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101001945CC36234B18439988D70FCB761011" ma:contentTypeVersion="11" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="49d1d5a573ca54dccef2d71c1bfe4d0c">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="36cf0646-7300-4608-bcc3-e29ed014863a" xmlns:ns3="734bc881-a844-4d86-9741-49f87248cc41" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fb428a4efaeddf2ef8bccbe6d8f13bc5" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101001945CC36234B18439988D70FCB761011" ma:contentTypeVersion="11" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="8ca733e0ec3c0df6e34813901e7a3ca5">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="36cf0646-7300-4608-bcc3-e29ed014863a" xmlns:ns3="734bc881-a844-4d86-9741-49f87248cc41" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="aed9a3083501fe1d9ea761da13b3b1bf" ns2:_="" ns3:_="">
     <xsd:import namespace="36cf0646-7300-4608-bcc3-e29ed014863a"/>
     <xsd:import namespace="734bc881-a844-4d86-9741-49f87248cc41"/>
     <xsd:element name="properties">
@@ -1087,24 +1130,26 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="36cf0646-7300-4608-bcc3-e29ed014863a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="734bc881-a844-4d86-9741-49f87248cc41" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD571DE7-56CF-4046-837C-EA8124263E5D}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C2DBC01-C33C-446B-9484-7BA7D14E7651}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC422C81-0F6E-45C7-8ED1-45D7A93F939C}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{557E2686-30D3-4FF3-8CA9-B4A39B1B1B1E}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD571DE7-56CF-4046-837C-EA8124263E5D}"/>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>